<commit_message>
Leads: 2026-10-06 01:24 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>abileneappliancerepairtx.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>abileneappliancerepairtx.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://abileneappliancerepairtx.com/services/water-heater-repair-abilene/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>contact.appliancerepairabilene@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3253390690</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>water heater repair Abilene TX</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 01:26 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://abileneappliancerepairtx.com/services/water-heater-repair-abilene/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>contact.appliancerepairabilene@gmail.com</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Meridian Idaho Roofing Company | Residential &amp; Commercial Roofers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>nwroof.net</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://nwroof.net/service-area/roofers-meridian-idaho-commercial-residential</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Shingle Roofing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@nwroof.net</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>208-440-2205</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roof repair company Meridian ID</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 01:29 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Cranston RI | GT Restoration</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>gtrestoration.us</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.gtrestoration.us/pbs/roofing-contractor-in-rhode-island-cranston-ri</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rhode Island</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@gtrestoration.us</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(401) 405-9083</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Cranston RI</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor Cranston RI</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 01:34 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Quality Aurora AC Repair</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>qualityauroraacrepair.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>http://qualityauroraacrepair.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mark Stevens</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@qualityauroraacrepair.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(720) 796-7762</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>72</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>air conditioning repair Aurora CO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:10 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,126 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ONEWAY ROOFING</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>onewayroof.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://onewayroof.com/service-areas/st-charles-county/o-fallon/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Roof Quote</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@onewayroof.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(314) 209-1782</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roofing contractor OFallon MO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Black Roofing &amp; Waterproofing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>blackroofing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://blackroofing.com/service-area/arvada-co/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Why Arvada</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@blackroofing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(303) 449-5176</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>94</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roofing contractor Arvada CO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:12 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Anchor Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>anchorplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://anchorplumbingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Highland Park</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>johnsmith@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(214) 946-1638</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>plumbing company Dallas TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:18 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADN Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>adnroofingct.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.adnroofingct.com/roofers-stamford-ct/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fully Licensed</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@adnroofingct.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(203) 751-3091</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Stamford CT</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:22 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,122 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Provo Plumber | MAC Plumbing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>macplumbingutah.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.macplumbingutah.com/provo-plumber</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>American Fork</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>macplumbingheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(801) 361-6842</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Provo UT</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>plumbing company Provo UT</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Von Eric Roofing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>vonericroofing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://vonericroofing.com/broken-arrow/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@vonericroofing.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>918-361-1786</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roof replacement Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:27 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,6 @@
           <t>https://vonericroofing.com/broken-arrow/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@vonericroofing.com</t>
@@ -1149,6 +1148,62 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Heating &amp; Cooling Experts – Portland, OR – Rose Heating</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>roseheating.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.roseheating.com/portland-hvac-company-or</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>roseheating@earthlink.net</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(503) 283-5183</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>heating and cooling company Portland OR</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:29 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1174,7 +1174,6 @@
           <t>https://www.roseheating.com/portland-hvac-company-or</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>roseheating@earthlink.net</t>
@@ -1204,6 +1203,62 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fremont Heating &amp; Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>fremonthvac.net</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.fremonthvac.net/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>service@fremonthavac.net</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(801) 920-6377</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ogden UT</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:31 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1229,7 +1229,6 @@
           <t>https://www.fremonthvac.net/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>service@fremonthavac.net</t>
@@ -1259,6 +1258,122 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Adaquate A/C &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>adaquate.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://adaquate.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>lorenzo@adaquate.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(432) 653-5164</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>98</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>AC installation Odessa TX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Colorado Springs &amp; El Paso County HVAC | Springs Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>springshac.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://springshac.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>View Financing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@springsheating.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(719) 235-3779</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>HVAC contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:38 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1284,6 @@
           <t>https://adaquate.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>lorenzo@adaquate.com</t>
@@ -1374,6 +1373,66 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Yeti Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>hvacyeti.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://hvacyeti.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Yeti Heating</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>sales@hvacyeti.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>717.942.1104</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>heating and cooling company York PA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:44 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1438,6 +1438,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Local Roofing &amp; Construction — Federal Way, WA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>localroofingconstruction.net</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://localroofingconstruction.net/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Start My</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>contact@localroofingconstruction.net</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(206) 931-4986</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roofing contractor Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:48 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1498,6 +1498,122 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C &amp; L Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>derbycityhvac.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.derbycityhvac.com/heat-pump-replacement-louisville-ky/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@derbycityhvac.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(502) 969-7016</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>heat pump installation Louisville KY</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Louisville KY | Buehner HVAC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>buehnerhvac.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://buehnerhvac.com/hvac-services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Blog Privacy</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>service@buehnerhvac.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(502) 604-9122</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>heat pump installation Louisville KY</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:50 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1519,7 +1519,6 @@
           <t>https://www.derbycityhvac.com/heat-pump-replacement-louisville-ky/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>info@derbycityhvac.com</t>
@@ -1609,6 +1608,122 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Handy Manny's LLC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>handymannysky.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://handymannysky.com/locations/roofing-contractor-lexington-ky</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Development Services</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>manny@handymannys.biz</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(859) 551-5302</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roofing contractor Lexington KY</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Butler Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>butlerroofingky.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.butlerroofingky.com/roofing-lexington-ky</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Serve Yours</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@butlerroofingky.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>76</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>roofing contractor Lexington KY</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:52 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1704,7 +1704,6 @@
           <t>info@butlerroofingky.com</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Lexington KY</t>
@@ -1724,6 +1723,66 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Powell &amp; Sons Roofing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>powellandsonsroofing.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://powellandsonsroofing.com/service-areas/gainesville-fl</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sons Roofing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>powellandsonsroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(386) 294-1755</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roof replacement Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 11:59 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1788,6 +1788,62 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Pro</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>draincleaningpro.us</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://draincleaningpro.us/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>draincleaningpro.us@gmail.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(917) 914-6525</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>94</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>drain cleaning service New York NY</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:01 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1809,7 +1809,6 @@
           <t>https://draincleaningpro.us/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>draincleaningpro.us@gmail.com</t>
@@ -1839,6 +1838,178 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cobra Rooter &amp; Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>cobrarooter.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.cobrarooter.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Frequently Asked</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>jerrycrp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(480) 897-9211</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>plumbing company Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Desert Valley Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>desertvalleyhvac.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://desertvalleyhvac.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Blue Diamond</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>office@desertvalleyhvac.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(702) 539-2801</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Henderson NV</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>heating and cooling company Henderson NV</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Paar Plumbing</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>paarplumbing.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://paarplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>mike@paarplumbing.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>64</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>plumbing company Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:03 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1984,13 +1984,11 @@
           <t>https://paarplumbing.com/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>mike@paarplumbing.com</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Phoenix AZ</t>
@@ -2010,6 +2008,62 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Plumbing and Heating Repair - Casper, WY - Huber Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>plumbingcasper.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.plumbingcasper.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>huberplumb@aol.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>307-234-3851</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>plumber Casper WY</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:06 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2034,7 +2034,6 @@
           <t>https://www.plumbingcasper.com/</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>huberplumb@aol.com</t>
@@ -2064,6 +2063,62 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CJ Roofing, LLC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>cjroofingdc.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://cjroofingdc.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>cj.roofing.dc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>202-770-4971</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>96</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roofing contractor Washington DC</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:08 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2089,7 +2089,6 @@
           <t>https://cjroofingdc.com/</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>cj.roofing.dc@gmail.com</t>
@@ -2119,6 +2118,62 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Weikle's Hometown Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>weikleshometownhvac.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://weikleshometownhvac.com/areas-we-serve/wilmington-nc/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@weikleshometownhvac.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>910-931-0094</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>heating and cooling company Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:12 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2144,7 +2144,6 @@
           <t>https://weikleshometownhvac.com/areas-we-serve/wilmington-nc/</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>info@weikleshometownhvac.com</t>
@@ -2174,6 +2173,182 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Indianapolis, IN</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ayresmechanicalinc.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://ayresmechanicalinc.com/services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>info@ayresmechanicalinc.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(317) 342-9345</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>heat pump installation Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Bowman's Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>bowmansheatingandcooling.net</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://bowmansheatingandcooling.net/services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Cooling Fast</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>service@bowmansheatingandcooling.net</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(317) 449-8745</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>heat pump installation Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Roof Repair, Replacement &amp; Leak Repair in Coral Springs | D&amp;Co Homes</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>dandcohomes.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.dandcohomes.com/roofing-coral-springs</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Dwelling Units</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>office@dandcohomes.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(561) 983-5344</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>roof repair company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:23 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2199,7 +2199,6 @@
           <t>https://ayresmechanicalinc.com/services/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>info@ayresmechanicalinc.com</t>
@@ -2349,6 +2348,126 @@
         </is>
       </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>KangaRoof</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>callkangaroof.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://callkangaroof.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Get Instant</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@callkangaroof.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(512) 388-7663</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>100</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>roof replacement Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Efficient AC, Electric &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>efficienttexas.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://efficienttexas.com/new-braunfels/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Owners George</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>kate@efficienttexas.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>512-501-2275</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>HVAC contractor New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:27 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2473,6 +2473,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Precision Plumbers Nampa</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>precisionplumbersnampa.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://precisionplumbersnampa.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@precisionplumbersnampa.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(208) 318-5818</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Nampa ID</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>emergency plumber Nampa ID</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:34 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2494,7 +2494,6 @@
           <t>https://precisionplumbersnampa.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>info@precisionplumbersnampa.com</t>
@@ -2524,6 +2523,126 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>North TX HVAC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>northtxhvac.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.northtxhvac.com/service-area/grand-prairie/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cooling Experts</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>bryan@northtxhvac.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>817-717-1855</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>HVAC contractor Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Welch Plumbing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>welchplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.welchplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Welch Plumbing</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>welchplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(318) 507-8035</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Shreveport LA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>90</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>plumbing company Shreveport LA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:36 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2648,6 +2648,242 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Roofers | Naperville, IL | Fritz Roofing Service Inc</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>fritzroofingservices.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.fritzroofingservices.com/contact/roofers-service-area/naperville-il</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Fritz Roofing</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@fritzroofingservices.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(847) 641-4155</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>roofing contractor Naperville IL</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Naperville IL Roofers</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>maxroofings.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://maxroofings.com/naperville-il-roofers/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Roofing Services</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>contact@maxroofings.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>773.766.9988</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>roofing contractor Naperville IL</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HVAC Services Riverside, CA | Steve's Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>stevesairconditioningandheating.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://stevesairconditioningandheating.com/service-areas/riverside-ca</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Why Neighbors</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>stevesac_6708@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>9516343233</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>90</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>air conditioning repair Riverside CA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>The Drain Guys</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>thedrainguysidaho.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.thedrainguysidaho.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>208.921.2263</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>82</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>drain cleaning service Boise ID</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:44 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2849,7 +2849,6 @@
           <t>https://www.thedrainguysidaho.com/</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>example@mysite.com</t>
@@ -2879,6 +2878,66 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Plumbers, Heating</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>allen-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.allen-plumbing.com/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Note From</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>info@allen-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(617) 625-4300</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>78</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>plumber Boston MA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:46 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2943,6 +2943,182 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cinnamon Energy Systems</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>cinnamon.energy</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://cinnamon.energy/hvac/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>info@cinnamon.energy</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(408) 883-7000</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>100</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>heat pump installation Metairie LA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Pipes R Us Plumbing</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>pipesrusnola.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://pipesrusnola.com/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Danny Griffin</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>pipesrusplumbing2010@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>504-866-2730</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>plumber New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SVCE</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>svcleanenergy.org</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.svcleanenergy.org/heatpumps/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sybil Cramer</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>info@svcleanenergy.org</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>86</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>heat pump installation Metairie LA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:53 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3094,7 +3094,6 @@
           <t>info@svcleanenergy.org</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>Metairie LA</t>
@@ -3114,6 +3113,66 @@
         </is>
       </c>
       <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>AC Remedies</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>acremedies.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://acremedies.com/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>List Super</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@acremedies.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>601-238-2509</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Jackson MS</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>76</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>AC installation Jackson MS</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:55 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3178,6 +3178,62 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Brothers Metal Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>brothersmetalroofing.net</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://brothersmetalroofing.net/service-area/ohio/dayton/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@brothersmetalroofing.net</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(937) 423-9352</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>86</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Dayton OH</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:57 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3199,7 +3199,6 @@
           <t>https://brothersmetalroofing.net/service-area/ohio/dayton/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>info@brothersmetalroofing.net</t>
@@ -3229,6 +3228,66 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Idaho Roofing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>idahoroofing.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://idahoroofing.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Eastern Idaho</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>justroofit101@gmail.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(208) 317-5571</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>90</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roofing contractor Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 12:59 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3293,6 +3293,118 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Miracle</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>miracleplumbing.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.miracleplumbing.com/services/heating-and-cooling/heat-pump-installation-repair/akron/oh</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@miracle1927.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>330-773-4499</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>heat pump installation Akron OH</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair &amp; Replacement | Smooth Plumbing</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>smoothplumbingfl.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://smoothplumbingfl.com/services/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>info@smoothplumbingfl.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>239-888-7667</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>sewer repair Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:01 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3314,7 +3314,6 @@
           <t>https://www.miracleplumbing.com/services/heating-and-cooling/heat-pump-installation-repair/akron/oh</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>info@miracle1927.com</t>
@@ -3370,7 +3369,6 @@
           <t>https://smoothplumbingfl.com/services/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>info@smoothplumbingfl.com</t>
@@ -3400,6 +3398,66 @@
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Southern Traditions Roofing</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>southern-traditions-roofing.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.southern-traditions-roofing.com/roofing/palm-bay-fl</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>August Pleveich</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>apleveich@southern-traditions-roofing.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(407) 579-6397</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>roofing contractor Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:05 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3463,6 +3463,66 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Plumbing Fixture, Water Heater &amp; Gas Line Installation | Rogers, Bentonville, Fa</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>plumbbrokeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.plumbbrokeplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>No Drip</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>plumbbroke2024@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(855) 463-5490</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>86</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>plumbing company Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:12 UTC (cycle 67)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3523,6 +3523,122 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Weiss Air Conditioning and Plumbing</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>weissacandheat.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://weissacandheat.com/conroe-ac-plumbing/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Weiss Air</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>hello@justcallweiss.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(281) 936-8216</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>air conditioning repair Conroe TX</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Ritter's Roofing</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>rittersroofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://rittersroofing.com/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>rittersroofingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(570) 335-1483</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Scranton PA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>88</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>roof repair company Scranton PA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:14 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3604,7 +3604,6 @@
           <t>https://rittersroofing.com/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>rittersroofingllc@gmail.com</t>
@@ -3634,6 +3633,66 @@
         </is>
       </c>
       <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Best Marietta Roofer</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>bestmariettaroofer.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://bestmariettaroofer.com/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>bestmariettaroofer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(470) 777-7344</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>100</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roofer Marietta GA</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:16 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3698,6 +3698,66 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Burkholder's Heating &amp; Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>burkholders-hvac.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.burkholders-hvac.com/residential-hvac-services/residential-air-conditioning/residential-ac-installations/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Bob Burkholder</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>service@burkhvac.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>610-816-6889</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Allentown PA</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>AC installation Allentown PA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:20 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3758,6 +3758,66 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Ohio Water Heater Authority</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ohiowaterheaterauthority.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://ohiowaterheaterauthority.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Flow Group</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>hello@ohiowaterheaterauthority.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>844-792-8374</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>100</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>water heater repair Columbus OH</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:26 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3818,6 +3818,62 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Cornerstone Pros</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>cornerstonepros.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://cornerstonepros.com/plumbing-services/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>service@cornerstonepros.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(813) 921-2610</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>100</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>water heater repair Tampa FL</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:27 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3839,7 +3839,6 @@
           <t>https://cornerstonepros.com/plumbing-services/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>service@cornerstonepros.com</t>
@@ -3869,6 +3868,242 @@
         </is>
       </c>
       <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>360 Power Roofing</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>360powerroofing.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://360powerroofing.com/roofing-company-the-woodlands-tx/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Power Roofing</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>info@360powerroofing.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>832-246-9931</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>residential roofing company The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>HVAC in Meridian &amp; Boise, ID</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>meridianhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://meridianhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Treasure Valley</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>hello@meridianhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(555) 000-0000</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>HVAC contractor Meridian ID</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ROYH Build Co</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>royhbuildco.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.royhbuildco.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Build Co</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>info@royhbuildco.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(281) 825-8385</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>residential roofing company The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Taylor Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>taylorheatingandairva.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://taylorheatingandairva.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>wtaylor@taylorconstructionservices.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>804-271-7776</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>90</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>HVAC contractor Richmond VA</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:29 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4074,7 +4074,6 @@
           <t>https://taylorheatingandairva.com/</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>wtaylor@taylorconstructionservices.com</t>
@@ -4104,6 +4103,66 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Roofing Company in Cedar Rapids, IA | Roof Replacement &amp; Repair | Passion Exteri</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>passionexteriors.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.passionexteriors.com/service-areas/cedar-rapids</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Gutters Learn</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>admin@passionexteriors.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>319-536-1924</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>roof repair company Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:31 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4168,6 +4168,66 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Omaha Plumbing Pro</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>omahaplumbing.pro</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://omahaplumbing.pro/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@omahaplumbing.pro</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(402) 538-8333</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>plumbing company Omaha NE</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:33 UTC (cycle 78)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4228,6 +4228,62 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Roofing Contractor | High Point, NC | Well Done Roofing</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>welldoneroofingofnc.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.welldoneroofingofnc.com/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>welldoneroofing2014@gmail.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(336) 905-0476</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>86</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>roofing contractor High Point NC</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:41 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4249,7 +4249,6 @@
           <t>https://www.welldoneroofingofnc.com/</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>welldoneroofing2014@gmail.com</t>
@@ -4279,6 +4278,62 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Hawkeye Roofing 1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>hawkeyeroofs.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.hawkeyeroofs.com/locations/durham</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>treine@hawkeyeroofs.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>919-727-4295</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>residential roofing company Durham NC</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:43 UTC (cycle 83)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4304,7 +4304,6 @@
           <t>https://www.hawkeyeroofs.com/locations/durham</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>treine@hawkeyeroofs.com</t>
@@ -4334,6 +4333,66 @@
         </is>
       </c>
       <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Granite Mountain Roofing</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>granitemtroofing.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://granitemtroofing.com/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Shane Jordan</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>sales@granitrmtroofing.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>509-850-8987</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>100</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>roofing contractor Spokane WA</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:45 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4398,6 +4398,66 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Bauer Mechanical Services HVAC | Serving Fort Collins, CO</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>bauermechanicalhvac.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://bauermechanicalhvac.com/fort-collins</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Bauer Mechanical</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>matthew.siemens@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(970) 373-0381</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>90</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:50 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4458,6 +4458,62 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Annapolis, MD</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>410newroof.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://410newroof.com/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>sales@410newroof.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(410) 639-7663</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roof replacement Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 13:52 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4479,7 +4479,6 @@
           <t>https://410newroof.com/roof-replacement/</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>sales@410newroof.com</t>
@@ -4509,6 +4508,122 @@
         </is>
       </c>
       <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Furnace Pro</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>furnaceprohvac.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://furnaceprohvac.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>sebastian@aldusleaf.org</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>319-440-6399</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>88</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>furnace repair Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>gomezroofing-inc.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://gomezroofing-inc.com/home/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Gomez Roofing</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@gomezroofing-inc.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>775-220-4668</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>76</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>roof repair company Reno NV</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:01 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4534,7 +4534,6 @@
           <t>https://furnaceprohvac.com/</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>sebastian@aldusleaf.org</t>
@@ -4624,6 +4623,62 @@
         </is>
       </c>
       <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Capstone Plumbing</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>capstoneplumbing.net</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://capstoneplumbing.net/drain-cleaning-birmingham-al/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>serviceteam@capstoneplumbing.net</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>205-434-7224</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>drain cleaning service Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:12 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4649,7 +4649,6 @@
           <t>https://capstoneplumbing.net/drain-cleaning-birmingham-al/</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>serviceteam@capstoneplumbing.net</t>
@@ -4679,6 +4678,62 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Expert Plumbers in Pembroke Pines, FL</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>plumbersofpembrokepines.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://plumbersofpembrokepines.com/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>gr8american@comcast.net</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(954) 578-1080</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>90</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>emergency plumber Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:14 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4704,7 +4704,6 @@
           <t>https://plumbersofpembrokepines.com/</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>gr8american@comcast.net</t>
@@ -4734,6 +4733,66 @@
         </is>
       </c>
       <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AC Repair Miami, FL | Air Temp Service</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>airtempmiami.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.airtempmiami.com/ac-repair</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>airtemp@live.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(305) 436-2801</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>90</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>air conditioning repair Miami FL</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:16 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4798,6 +4798,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Cregger Plumbing, Heating, Cooling &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>creggerplumbing.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.creggerplumbing.com/service-area-livonia/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Metro Detroit</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>creggeroffice@creggerphc.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>248-543-1190</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Livonia MI</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>emergency plumber Livonia MI</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:18 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4858,6 +4858,122 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>EZ Plumbing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ez-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://ez-plumbing.com/residential-plumbing/drain-cleaning/drain-cleaning-los-angeles/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Plumbing Focuses</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>service1@ez-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(818) 908-2710</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>90</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>drain cleaning service Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Team Rooter Plumbing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>teamrooter.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.teamrooter.com/drain-sewer/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>info@teamrooter.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(800) 818-2397</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>90</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>drain cleaning service Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:26 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4939,7 +4939,6 @@
           <t>https://www.teamrooter.com/drain-sewer/</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>info@teamrooter.com</t>
@@ -4969,6 +4968,62 @@
         </is>
       </c>
       <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>PlumbTechPros - Smart Solutions for Every Plumbing Need</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>plumbtechpros.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.plumbtechpros.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>plumber@plumbtechpros.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(800) 388-8149</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>100</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>plumber San Diego CA</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:28 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4994,7 +4994,6 @@
           <t>https://www.plumbtechpros.com/</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>plumber@plumbtechpros.com</t>
@@ -5024,6 +5023,62 @@
         </is>
       </c>
       <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DFW Roofing Pro</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>dfwroofingpro.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://dfwroofingpro.com/contact-us/irving-tx-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>contact@dfwroofingpro.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(972) 979-1070</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Irving TX</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>90</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>residential roofing company Irving TX</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:32 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5049,7 +5049,6 @@
           <t>https://dfwroofingpro.com/contact-us/irving-tx-roofing-company/</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>contact@dfwroofingpro.com</t>
@@ -5079,6 +5078,66 @@
         </is>
       </c>
       <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Jay’s Plumbing &amp; Services</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>jaysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://jaysplumbing.com/north-las-vegas-plumber/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>North Las</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>service@jaysplumbing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(702) 871-7488</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>90</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>plumbing company North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:39 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5143,6 +5143,126 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Freon Service</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>freonhvac.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.freonhvac.com/service-areas/heating-and-air-conditioning-fremont-ca/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Conditioning Service</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>install@freonhvac.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(408) 877-5557</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>100</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>heating and cooling company Fremont CA</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Rocky Top Roofing Inc.</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>rockytoproofing.net</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://rockytoproofing.net/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Star Reviews</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>danny@rockytoproofing.net</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>423-693-7286</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>76</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>roofing contractor Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:41 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5263,6 +5263,126 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>5Star Plumbing Salinas</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>5starplumbingsalinas.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://5starplumbingsalinas.com/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>East Salinas</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>info@5starplumbingsalinas.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(831) 279-2474</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>plumbing company Salinas CA</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>All Weather Roofing</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>nobuckets.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://nobuckets.com/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Roofing Contracts</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@nobuckets.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(209) 474-0258</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>86</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>residential roofing company Stockton CA</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 14:56 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5383,6 +5383,122 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Schultz Roofing Co</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>schultzroofingco.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.schultzroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>admin@schultzroofingco.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(904)246-2315</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>90</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>residential roofing company Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Alta Roofing</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>altaroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.altaroofingpros.com/service-areas/san-marcos</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Operated Roofer</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>info@altaroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(737) 260-7765</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>roofing contractor San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:07 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5404,7 +5404,6 @@
           <t>https://www.schultzroofingco.com/</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>admin@schultzroofingco.com</t>
@@ -5494,6 +5493,66 @@
         </is>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Sitton Roofing Co</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>sittonroof.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://sittonroof.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Why More</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>sittonroofing.co@gmail.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(325) 677-5416</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>98</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Abilene TX</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:09 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5558,6 +5558,62 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation and Replacement in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>contact@centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(833) 435-6630</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>heat pump installation Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:11 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5579,7 +5579,6 @@
           <t>https://aberdeen-sd.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>contact@centralheatairconditioning.com</t>
@@ -5609,6 +5608,126 @@
         </is>
       </c>
       <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Quality Air Services</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>qualityairservices.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://qualityairservices.com/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Metro Area</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>sales@qualityairservices.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>301-495-9500</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>100</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>HVAC contractor Washington DC</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Fortiz Hvac</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>fortizhvac.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://fortizhvac.com/washington-dc-hvac-contractor/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Mission At</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>fortizhvacinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(240) 573-6584</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>HVAC contractor Washington DC</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:13 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5733,6 +5733,62 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>AC Installation Services in Houston, TX</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>championandnash.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://championandnash.com/services/ac/ac-install</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>info@championandnash.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>713.997.8495</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>AC installation Houston TX</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:15 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5754,7 +5754,6 @@
           <t>https://championandnash.com/services/ac/ac-install</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>info@championandnash.com</t>
@@ -5784,6 +5783,182 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Residential Roofing in Flint, MI | Call Sweers Roofing</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>sweersroofing.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.sweersroofing.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Shingle Roofing</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>admin@sweersroofing.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(810) 743-2759</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Flint MI</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>90</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>residential roofing company Flint MI</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>freds-plumbing</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>fredsplumbingmt.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.fredsplumbingmt.com/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>fredsplb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(406) 543-7622</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>plumber Missoula MT</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Flash Roofing &amp; Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>flashroofingmiami.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.flashroofingmiami.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Flash Roofing</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>flashroofingmiami@gmail.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(786) 237-9440</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>90</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Miami FL</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:18 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5869,7 +5869,6 @@
           <t>https://www.fredsplumbingmt.com/</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>fredsplb@gmail.com</t>
@@ -5959,6 +5958,118 @@
         </is>
       </c>
       <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Forge Construction Group</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forgecg.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.forgecg.com/durham/roofing-services/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>keenan@forgecg.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(984) 369-9802</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>90</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>roofing contractor Durham NC</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Plumbing Innovators</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>plumbinginnovators.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.plumbinginnovators.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>janesmith@mail.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>540-679-7608</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>90</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>plumbing company Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:24 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5984,7 +5984,6 @@
           <t>https://www.forgecg.com/durham/roofing-services/</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>keenan@forgecg.com</t>
@@ -6040,7 +6039,6 @@
           <t>https://www.plumbinginnovators.com/</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>janesmith@mail.com</t>
@@ -6070,6 +6068,126 @@
         </is>
       </c>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Lafayette Plumbing Company | CJ's Plumbing Repair</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>cjsplumbingandrepair.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.cjsplumbingandrepair.com/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Residential See</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>cjplumbingrepair@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(337) 234-9769</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>100</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>plumbing company Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Roof Repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>roofrepairpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.roofrepairpasadenatx.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>info@roofrepairpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(346) 783-0077</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>90</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>roof repair company Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:32 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6193,6 +6193,66 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Missouri Heat Pump Installation</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>missouriheatpumpinstall.shop</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://missouriheatpumpinstall.shop/locations/ofallon/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Heat Pump</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>team@missouriheatpumpinstall.shop</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(314) 784-0963</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>100</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>heat pump installation OFallon MO</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:34 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6253,6 +6253,62 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Roofers | Lehi, UT | Pro Contractors Co LLC</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>proroofingutah.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.proroofingutah.com/contact/roofers-service-area/lehi-ut</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>procontractorsco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(385) 218-0527</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>roofer Lehi UT</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:37 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6274,7 +6274,6 @@
           <t>https://www.proroofingutah.com/contact/roofers-service-area/lehi-ut</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>procontractorsco@gmail.com</t>
@@ -6304,6 +6303,62 @@
         </is>
       </c>
       <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Weather Makers Queens</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>weathermakersqueens.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://weathermakersqueens.com/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>info@weathermakersqueens.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(516) 853-4535</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>AC installation Queens NY</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:41 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6329,7 +6329,6 @@
           <t>https://weathermakersqueens.com/</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>info@weathermakersqueens.com</t>
@@ -6359,6 +6358,186 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>German Roofing</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>germanroofing.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://germanroofing.com/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>German Roofing</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>hello@germanroofing.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>480-370-0300</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>roofing contractor Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Redemption Roofing AZ | Mesa &amp; Phoenix Roofing Contractor | Roof Repair &amp; Replac</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>redemptionroofingaz.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://redemptionroofingaz.com/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Google Miki</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>info@redemptionroofingaz.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(480) 920-2000</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>roofing contractor Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Blackstone Roofing Group</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>blackstoneroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://blackstoneroofinggroup.com/mesa/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>office@blackstoneroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(602) 536-9363</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>90</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>roofing contractor Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:47 UTC (cycle 149)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6543,6 +6543,66 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Rampart Roofing Colorado</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>rampartroofing.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://rampartroofing.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Hail Damage</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>info@rampartroofing.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>719-487-7663</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>100</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>roofer Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:51 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6603,6 +6603,122 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Chief Roofers Kansas City</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>chiefrooferskansascity.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://chiefrooferskansascity.com/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Commercial Roofi</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>info@chiefrooferskansascity.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(913) 553-4072</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Kansas City MO</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>roofer Kansas City MO</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>I &amp; J Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>iandjplumbing.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://iandjplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@iandjplumbing.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(954) 249 6278</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>plumbing company Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:52 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6684,7 +6684,6 @@
           <t>https://iandjplumbing.com/</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>info@iandjplumbing.com</t>
@@ -6714,6 +6713,66 @@
         </is>
       </c>
       <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Roofing Company in New Braunfels, TX | Compass Roofing Services</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>compassroofpros.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://compassroofpros.com/roofing-new-braunfels-tx</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Commercial We</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@compassroofpros.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>210-328-2127</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>86</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>residential roofing company New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:54 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6778,6 +6778,66 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Valle's Plumbing &amp; Rooter</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>vallesplumbingandrooter.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://vallesplumbingandrooter.com/services/sewer-line-repair-san-jose/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Get Free</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>valle862@gmail.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(408) 840-5932</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>San Jose CA</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>100</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>sewer repair San Jose CA</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 15:58 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6838,6 +6838,66 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Stellar Roofing Company</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>roofstellar.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.roofstellar.com/guide/best-metal-roofing-contractors-in-grand-rapids</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Paul Aikens</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>info@roofstellar.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(616) 840-1927</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>100</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 16:00 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6898,6 +6898,122 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Plumbing Company | Chesapeake, VA | Lanthorn Plumbing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>lanthornplumbingva.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.lanthornplumbingva.com/contact/plumbing-company-service-area/chesapeake-va</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>lanthornplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(757) 384-0021</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>100</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>plumbing company Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>York, PA Roofing</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>crainroofing.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://crainroofing.com/york</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Master Elite</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@crainroofing.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(717) 574-2652</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>90</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofer York PA</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-06 18:10 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6919,7 +6919,6 @@
           <t>https://www.lanthornplumbingva.com/contact/plumbing-company-service-area/chesapeake-va</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>lanthornplumbing@gmail.com</t>
@@ -7009,6 +7008,62 @@
         </is>
       </c>
       <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Commercial HVAC &amp; Mechanical Contractor Waukesha WI | Bredan Mechanical Systems</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>bredanmech.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://bredanmech.com/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>info@bredanmech.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>262-521-9919</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Waukesha WI</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>HVAC contractor Waukesha WI</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 18:13 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7034,7 +7034,6 @@
           <t>https://bredanmech.com/</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>info@bredanmech.com</t>
@@ -7064,6 +7063,62 @@
         </is>
       </c>
       <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Metal roofing in Grand Prairie Estates, Grand Prairie</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>dallasroofrepaircontractors.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://dallasroofrepaircontractors.com/locations/grand-prairie-tx/metal-roofing/grand-prairie-estates</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>info@dallasroofrepaircontractors.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(972) 944-0485</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 18:14 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7089,7 +7089,6 @@
           <t>https://dallasroofrepaircontractors.com/locations/grand-prairie-tx/metal-roofing/grand-prairie-estates</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>info@dallasroofrepaircontractors.com</t>
@@ -7119,6 +7118,66 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Ann Arbor Plumber | Residential Plumbing &amp; Water Heaters</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>mitchtheplumber-mi.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.mitchtheplumber-mi.com/locations/ann-arbor-mi</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Ann Arbor</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>alex@mitchtheplumber.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>734-995-5063</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>plumber Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-06 18:29 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-06.xlsx
+++ b/output/leads_2026-10-06.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7183,6 +7183,62 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Lilac Roofing and Siding</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>lilacroofing.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://lilacroofing.com/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>davis@lilacroofing.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>585-450-1590</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>roofer Rochester NY</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>